<commit_message>
docs: agregado base de datos Kairos, inicio especificación CU09 y CU20
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -33,8 +33,7 @@
     <t>Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">git log --all --date=short --pretty=format:"%ad" | sort | uniq -c
-</t>
+    <t>git log --all --date=short --pretty=format:"%ad" | sort | uniq -c</t>
   </si>
   <si>
     <t xml:space="preserve">SUMA </t>
@@ -176,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="281086657"/>
-        <c:axId val="1016346186"/>
+        <c:axId val="1234996272"/>
+        <c:axId val="1977053363"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="281086657"/>
+        <c:axId val="1234996272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -232,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1016346186"/>
+        <c:crossAx val="1977053363"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1016346186"/>
+        <c:axId val="1977053363"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -310,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="281086657"/>
+        <c:crossAx val="1234996272"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -615,7 +614,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A32)</f>
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -804,10 +803,20 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="6"/>
+      <c r="A28" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B28" s="8">
+        <v>45948.0</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="6"/>
+      <c r="A29" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="B29" s="8">
+        <v>45951.0</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="6"/>

</xml_diff>

<commit_message>
(docs) nuevo código de estimacion
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="791235614"/>
-        <c:axId val="1549021873"/>
+        <c:axId val="1236070941"/>
+        <c:axId val="1771326078"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="791235614"/>
+        <c:axId val="1236070941"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1549021873"/>
+        <c:crossAx val="1771326078"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1549021873"/>
+        <c:axId val="1771326078"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="791235614"/>
+        <c:crossAx val="1236070941"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A32)</f>
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -828,7 +828,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="7">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B31" s="8">
         <v>45954.0</v>

</xml_diff>

<commit_message>
docs: casos de prueba e implementacion
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1236070941"/>
-        <c:axId val="1771326078"/>
+        <c:axId val="1822824744"/>
+        <c:axId val="1005491640"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1236070941"/>
+        <c:axId val="1822824744"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1771326078"/>
+        <c:crossAx val="1005491640"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1771326078"/>
+        <c:axId val="1005491640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1236070941"/>
+        <c:crossAx val="1822824744"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A32)</f>
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -835,10 +835,29 @@
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="6"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
+      <c r="A32" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B32" s="8">
+        <v>45956.0</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B33" s="8">
+        <v>45957.0</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B34" s="8">
+        <v>45958.0</v>
+      </c>
+    </row>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: Inicio de priorización 2da tanda, inicio especificacion CU21
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1822824744"/>
-        <c:axId val="1005491640"/>
+        <c:axId val="1840360186"/>
+        <c:axId val="42108178"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1822824744"/>
+        <c:axId val="1840360186"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1005491640"/>
+        <c:crossAx val="42108178"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1005491640"/>
+        <c:axId val="42108178"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1822824744"/>
+        <c:crossAx val="1840360186"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -852,7 +852,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B34" s="8">
         <v>45958.0</v>

</xml_diff>

<commit_message>
docs: especificacion CU21 finalizado, documentos actualizados 31-10
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1840360186"/>
-        <c:axId val="42108178"/>
+        <c:axId val="185222335"/>
+        <c:axId val="982093323"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1840360186"/>
+        <c:axId val="185222335"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42108178"/>
+        <c:crossAx val="982093323"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42108178"/>
+        <c:axId val="982093323"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1840360186"/>
+        <c:crossAx val="185222335"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -341,8 +341,8 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5715000" cy="3533775"/>
     <xdr:graphicFrame>

</xml_diff>

<commit_message>
docs: Priorizacion 2da tanda CU finalizada
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="185222335"/>
-        <c:axId val="982093323"/>
+        <c:axId val="888422294"/>
+        <c:axId val="318286330"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="185222335"/>
+        <c:axId val="888422294"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="982093323"/>
+        <c:crossAx val="318286330"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="982093323"/>
+        <c:axId val="318286330"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="185222335"/>
+        <c:crossAx val="888422294"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -613,8 +613,8 @@
         <v>45897.0</v>
       </c>
       <c r="C4" s="6">
-        <f>SUM(A3:A32)</f>
-        <v>92</v>
+        <f>SUM(A3:A50)</f>
+        <v>115</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -858,8 +858,22 @@
         <v>45958.0</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B35" s="8">
+        <v>45960.0</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B36" s="8">
+        <v>45961.0</v>
+      </c>
+    </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
     <row r="39" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: inicio documento casos de prueba de CU 07, 13, 14
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -175,11 +175,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="888422294"/>
-        <c:axId val="318286330"/>
+        <c:axId val="2076748409"/>
+        <c:axId val="178123860"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="888422294"/>
+        <c:axId val="2076748409"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="318286330"/>
+        <c:crossAx val="178123860"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="318286330"/>
+        <c:axId val="178123860"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="888422294"/>
+        <c:crossAx val="2076748409"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A50)</f>
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -868,16 +868,44 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3">
-        <v>2.0</v>
+        <v>6.0</v>
       </c>
       <c r="B36" s="8">
         <v>45961.0</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B37" s="8">
+        <v>45962.0</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B38" s="8">
+        <v>45963.0</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B39" s="8">
+        <v>45964.0</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B40" s="8">
+        <v>45965.0</v>
+      </c>
+    </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: casos de pruebas avanzados
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -170,16 +170,16 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Hoja 1'!$A$3:$A$40</c:f>
+              <c:f>'Hoja 1'!$A$3:$A$43</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="2076748409"/>
-        <c:axId val="178123860"/>
+        <c:axId val="726027585"/>
+        <c:axId val="557636952"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2076748409"/>
+        <c:axId val="726027585"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +231,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="178123860"/>
+        <c:crossAx val="557636952"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="178123860"/>
+        <c:axId val="557636952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +309,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2076748409"/>
+        <c:crossAx val="726027585"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A50)</f>
-        <v>124</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -900,15 +900,36 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3">
-        <v>2.0</v>
+        <v>12.0</v>
       </c>
       <c r="B40" s="8">
         <v>45965.0</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B41" s="8">
+        <v>45966.0</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B42" s="8">
+        <v>45967.0</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B43" s="8">
+        <v>45968.0</v>
+      </c>
+    </row>
     <row r="44" ht="15.75" customHeight="1"/>
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: inicio de manuales
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>A</t>
   </si>
@@ -37,6 +37,21 @@
   </si>
   <si>
     <t xml:space="preserve">SUMA </t>
+  </si>
+  <si>
+    <t>Estado del repositorio</t>
+  </si>
+  <si>
+    <t>cantidad de carpetas</t>
+  </si>
+  <si>
+    <t>git rev-list --all | while read commit; do git ls-tree -r --name-only $commit; done | sed 's/[^/]*$//' | sort -u | wc -l</t>
+  </si>
+  <si>
+    <t>cantidad de archivos</t>
+  </si>
+  <si>
+    <t>git rev-list --all | while read commit; do git ls-tree -r --name-only $commit; done | sort -u | wc -l</t>
   </si>
 </sst>
 </file>
@@ -165,21 +180,21 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'Hoja 1'!$B$3:$B$40</c:f>
+              <c:f>'Hoja 1'!$B$3:$B$60</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Hoja 1'!$A$3:$A$43</c:f>
+              <c:f>'Hoja 1'!$A$3:$A$60</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="726027585"/>
-        <c:axId val="557636952"/>
+        <c:axId val="293473843"/>
+        <c:axId val="1605901206"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="726027585"/>
+        <c:axId val="293473843"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -231,10 +246,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="557636952"/>
+        <c:crossAx val="1605901206"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="557636952"/>
+        <c:axId val="1605901206"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -309,7 +324,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="726027585"/>
+        <c:crossAx val="293473843"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -344,7 +359,7 @@
       <xdr:row>2</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5715000" cy="3533775"/>
+    <xdr:ext cx="6219825" cy="3838575"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="1710398839" name="Chart 1" title="Gráfico"/>
@@ -614,7 +629,7 @@
       </c>
       <c r="C4" s="6">
         <f>SUM(A3:A50)</f>
-        <v>143</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -784,6 +799,9 @@
       <c r="B25" s="8">
         <v>45944.0</v>
       </c>
+      <c r="F25" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="G25" s="9"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -793,6 +811,9 @@
       <c r="B26" s="8">
         <v>45946.0</v>
       </c>
+      <c r="F26" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="7">
@@ -801,6 +822,9 @@
       <c r="B27" s="8">
         <v>45947.0</v>
       </c>
+      <c r="F27" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="7">
@@ -809,6 +833,9 @@
       <c r="B28" s="8">
         <v>45948.0</v>
       </c>
+      <c r="F28" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="7">
@@ -817,6 +844,9 @@
       <c r="B29" s="8">
         <v>45951.0</v>
       </c>
+      <c r="F29" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="7">
@@ -924,16 +954,44 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="3">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="B43" s="8">
         <v>45968.0</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="B44" s="8">
+        <v>45969.0</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B45" s="8">
+        <v>45970.0</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="3">
+        <v>13.0</v>
+      </c>
+      <c r="B46" s="8">
+        <v>45971.0</v>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B47" s="8">
+        <v>45972.0</v>
+      </c>
+    </row>
     <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: actualización de documentos(cierre construcción y planificación post cursada)
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -190,11 +190,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="293473843"/>
-        <c:axId val="1605901206"/>
+        <c:axId val="1396265117"/>
+        <c:axId val="1478690587"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="293473843"/>
+        <c:axId val="1396265117"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -246,10 +246,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1605901206"/>
+        <c:crossAx val="1478690587"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1605901206"/>
+        <c:axId val="1478690587"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -324,7 +324,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="293473843"/>
+        <c:crossAx val="1396265117"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -356,10 +356,10 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6219825" cy="3838575"/>
+    <xdr:ext cx="7505700" cy="4638675"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="1710398839" name="Chart 1" title="Gráfico"/>
@@ -628,8 +628,8 @@
         <v>45897.0</v>
       </c>
       <c r="C4" s="6">
-        <f>SUM(A3:A50)</f>
-        <v>186</v>
+        <f>SUM(A3:A80)</f>
+        <v>302</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -799,9 +799,6 @@
       <c r="B25" s="8">
         <v>45944.0</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="G25" s="9"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -811,9 +808,6 @@
       <c r="B26" s="8">
         <v>45946.0</v>
       </c>
-      <c r="F26" s="3" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="7">
@@ -822,9 +816,6 @@
       <c r="B27" s="8">
         <v>45947.0</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="7">
@@ -833,9 +824,6 @@
       <c r="B28" s="8">
         <v>45948.0</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="7">
@@ -844,9 +832,6 @@
       <c r="B29" s="8">
         <v>45951.0</v>
       </c>
-      <c r="F29" s="3" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="7">
@@ -879,6 +864,9 @@
       <c r="B33" s="8">
         <v>45957.0</v>
       </c>
+      <c r="F33" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3">
@@ -887,6 +875,9 @@
       <c r="B34" s="8">
         <v>45958.0</v>
       </c>
+      <c r="F34" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3">
@@ -895,6 +886,9 @@
       <c r="B35" s="8">
         <v>45960.0</v>
       </c>
+      <c r="F35" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3">
@@ -903,6 +897,9 @@
       <c r="B36" s="8">
         <v>45961.0</v>
       </c>
+      <c r="F36" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="3">
@@ -911,6 +908,9 @@
       <c r="B37" s="8">
         <v>45962.0</v>
       </c>
+      <c r="F37" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="3">
@@ -986,21 +986,84 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="3">
-        <v>5.0</v>
+        <v>21.0</v>
       </c>
       <c r="B47" s="8">
         <v>45972.0</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
-    <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
-    <row r="55" ht="15.75" customHeight="1"/>
-    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="3">
+        <v>18.0</v>
+      </c>
+      <c r="B48" s="8">
+        <v>45973.0</v>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B49" s="8">
+        <v>45974.0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="B50" s="8">
+        <v>45975.0</v>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B51" s="8">
+        <v>45976.0</v>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B52" s="8">
+        <v>45977.0</v>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="B53" s="8">
+        <v>45978.0</v>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="3">
+        <v>19.0</v>
+      </c>
+      <c r="B54" s="8">
+        <v>45979.0</v>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="A55" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B55" s="8">
+        <v>45980.0</v>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="3">
+        <v>11.0</v>
+      </c>
+      <c r="B56" s="8">
+        <v>45981.0</v>
+      </c>
+    </row>
     <row r="57" ht="15.75" customHeight="1"/>
     <row r="58" ht="15.75" customHeight="1"/>
     <row r="59" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: inicio estructura de memoria del proyecto
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="F7ilNVVjraUfXZtVbzZsg/y6LFriwpu5ogKBGUZlYsk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="8u7A57w9g7ecO9LEvqLgIlNAKBelJsfuCUsa3Iepi5g="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>A</t>
   </si>
@@ -24,7 +24,7 @@
     <t>B</t>
   </si>
   <si>
-    <t>Comando</t>
+    <t>Comando cantidad de commits por día</t>
   </si>
   <si>
     <t>Cantidad</t>
@@ -34,6 +34,27 @@
   </si>
   <si>
     <t>git log --all --date=short --pretty=format:"%ad" | sort | uniq -c</t>
+  </si>
+  <si>
+    <t>Inicio - I1</t>
+  </si>
+  <si>
+    <t>Elaboración - I1</t>
+  </si>
+  <si>
+    <t>Elaboración - I2</t>
+  </si>
+  <si>
+    <t>Construcción - I1</t>
+  </si>
+  <si>
+    <t>Construcción - I2</t>
+  </si>
+  <si>
+    <t>Construcción - I3</t>
+  </si>
+  <si>
+    <t>Cierre</t>
   </si>
   <si>
     <t xml:space="preserve">SUMA </t>
@@ -53,15 +74,56 @@
   <si>
     <t>git rev-list --all | while read commit; do git ls-tree -r --name-only $commit; done | sort -u | wc -l</t>
   </si>
+  <si>
+    <t>Fecha creación repo</t>
+  </si>
+  <si>
+    <t>Fecha actual</t>
+  </si>
+  <si>
+    <t>Dias totales:</t>
+  </si>
+  <si>
+    <t>Dias efectivos:</t>
+  </si>
+  <si>
+    <t>Commits de documentación (filtrados):</t>
+  </si>
+  <si>
+    <t>Documentación</t>
+  </si>
+  <si>
+    <t>Commits de programación (filtrados):</t>
+  </si>
+  <si>
+    <t>Programación</t>
+  </si>
+  <si>
+    <t>Commits de documentación (no filtrados):</t>
+  </si>
+  <si>
+    <t>Otros</t>
+  </si>
+  <si>
+    <t>Commits de programación (no filtrados):</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Otros (creación de ramas, actualización de repositorio, conflictos, etc)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="dd&quot;-&quot;mm&quot;-&quot;yy"/>
+    <numFmt numFmtId="165" formatCode="d/M/yyyy"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -73,6 +135,12 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -92,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -107,16 +175,31 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="166" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -135,21 +218,21 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="1">
+              <a:defRPr b="1" sz="2400">
                 <a:solidFill>
-                  <a:srgbClr val="757575"/>
+                  <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="1">
+              <a:rPr b="1" sz="2400">
                 <a:solidFill>
-                  <a:srgbClr val="757575"/>
+                  <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:rPr>
-              <a:t>Cantidad de Commits</a:t>
+              <a:t>Clasificación de Commits</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -158,184 +241,138 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Hoja 1'!$A$1:$A$2</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln cmpd="sng">
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="6D9EEB"/>
               </a:solidFill>
-            </a:ln>
-          </c:spPr>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="6AA84F"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E06666"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:txPr>
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr lvl="0">
+                    <a:defRPr sz="2400"/>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr lvl="0">
+                    <a:defRPr i="0" sz="2400"/>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:txPr>
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr lvl="0">
+                    <a:defRPr sz="1800"/>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Hoja 1'!$B$3:$B$60</c:f>
+              <c:f>'Hoja 1'!$H$53:$H$55</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Hoja 1'!$A$3:$A$60</c:f>
+              <c:f>'Hoja 1'!$I$53:$I$55</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1396265117"/>
-        <c:axId val="1478690587"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1396265117"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr lvl="0">
-                  <a:defRPr b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                  </a:rPr>
-                  <a:t>Fecha</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:spPr/>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr lvl="0">
-              <a:defRPr b="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1478690587"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1478690587"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="B7B7B7"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:minorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC">
-                  <a:alpha val="0"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:minorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr lvl="0">
-                  <a:defRPr b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                  </a:rPr>
-                  <a:t>Cantidad</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr lvl="0">
-              <a:defRPr b="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1396265117"/>
-      </c:valAx>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.7416872099767982"/>
+          <c:y val="0.21747967479674798"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
         <a:p>
           <a:pPr lvl="0">
-            <a:defRPr b="0">
+            <a:defRPr b="1" sz="2400">
               <a:solidFill>
                 <a:srgbClr val="1A1A1A"/>
               </a:solidFill>
@@ -355,14 +392,82 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9105900" cy="5553075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1710398839" name="Chart1" title="Gráfico">
+          <a:extLst>
+            <a:ext uri="GoogleSheetsCustomDataVersion1">
+              <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" pictureOfChart="1"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8963025" cy="5553075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="787707118" name="Chart2" title="Gráfico">
+          <a:extLst>
+            <a:ext uri="GoogleSheetsCustomDataVersion1">
+              <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" pictureOfChart="1"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1504950</xdr:colOff>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7505700" cy="4638675"/>
+    <xdr:ext cx="8210550" cy="5076825"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1710398839" name="Chart 1" title="Gráfico"/>
+        <xdr:cNvPr id="608345063" name="Chart 3" title="Gráfico"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -371,10 +476,44 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>619125</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4543425" cy="2847975"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="217464181" name="Chart4" title="Gráfico">
+          <a:extLst>
+            <a:ext uri="GoogleSheetsCustomDataVersion1">
+              <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" pictureOfChart="1"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
@@ -581,8 +720,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="5" width="12.63"/>
-    <col customWidth="1" min="6" max="6" width="45.13"/>
+    <col customWidth="1" min="1" max="3" width="12.63"/>
+    <col customWidth="1" min="4" max="4" width="26.63"/>
+    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="6" max="6" width="80.5"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -596,6 +737,9 @@
       <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="J1" s="3">
+        <v>25.0</v>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -608,6 +752,30 @@
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="J2" s="3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4">
@@ -617,7 +785,35 @@
         <v>45895.0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
+      </c>
+      <c r="K3" s="6">
+        <f t="shared" ref="K3:K11" si="2">$J$1-A3</f>
+        <v>17</v>
+      </c>
+      <c r="L3" s="7" t="str">
+        <f t="shared" ref="L3:Q3" si="1">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M3" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N3" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O3" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P3" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q3" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -627,9 +823,37 @@
       <c r="B4" s="5">
         <v>45897.0</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="8">
         <f>SUM(A3:A80)</f>
-        <v>302</v>
+        <v>307</v>
+      </c>
+      <c r="K4" s="6">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="L4" s="7" t="str">
+        <f t="shared" ref="L4:Q4" si="3">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M4" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N4" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O4" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P4" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q4" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -639,6 +863,34 @@
       <c r="B5" s="5">
         <v>45898.0</v>
       </c>
+      <c r="K5" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L5" s="7" t="str">
+        <f t="shared" ref="L5:Q5" si="4">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="4">
@@ -647,6 +899,34 @@
       <c r="B6" s="5">
         <v>45901.0</v>
       </c>
+      <c r="K6" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L6" s="7" t="str">
+        <f t="shared" ref="L6:Q6" si="5">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="4">
@@ -655,6 +935,34 @@
       <c r="B7" s="5">
         <v>45902.0</v>
       </c>
+      <c r="K7" s="6">
+        <f t="shared" si="2"/>
+        <v>22</v>
+      </c>
+      <c r="L7" s="7" t="str">
+        <f t="shared" ref="L7:Q7" si="6">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M7" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N7" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O7" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P7" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q7" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="4">
@@ -663,6 +971,34 @@
       <c r="B8" s="5">
         <v>45905.0</v>
       </c>
+      <c r="K8" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L8" s="7" t="str">
+        <f t="shared" ref="L8:Q8" si="7">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="4">
@@ -671,6 +1007,34 @@
       <c r="B9" s="5">
         <v>45907.0</v>
       </c>
+      <c r="K9" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L9" s="7" t="str">
+        <f t="shared" ref="L9:Q9" si="8">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="4">
@@ -679,6 +1043,34 @@
       <c r="B10" s="5">
         <v>45908.0</v>
       </c>
+      <c r="K10" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L10" s="7" t="str">
+        <f t="shared" ref="L10:Q10" si="9">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="4">
@@ -687,6 +1079,34 @@
       <c r="B11" s="5">
         <v>45909.0</v>
       </c>
+      <c r="K11" s="6">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="L11" s="7" t="str">
+        <f t="shared" ref="L11:Q11" si="10">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M11" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N11" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O11" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P11" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q11" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="4">
@@ -695,6 +1115,34 @@
       <c r="B12" s="5">
         <v>45911.0</v>
       </c>
+      <c r="K12" s="7" t="str">
+        <f t="shared" ref="K12:K58" si="12">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L12" s="6">
+        <f t="shared" ref="L12:L16" si="13">$J$1-$A12</f>
+        <v>23</v>
+      </c>
+      <c r="M12" s="7" t="str">
+        <f t="shared" ref="M12:Q12" si="11">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N12" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O12" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P12" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q12" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="4">
@@ -703,6 +1151,34 @@
       <c r="B13" s="5">
         <v>45912.0</v>
       </c>
+      <c r="K13" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L13" s="6">
+        <f t="shared" si="13"/>
+        <v>22</v>
+      </c>
+      <c r="M13" s="7" t="str">
+        <f t="shared" ref="M13:Q13" si="14">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N13" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O13" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P13" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q13" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="4">
@@ -711,6 +1187,34 @@
       <c r="B14" s="5">
         <v>45916.0</v>
       </c>
+      <c r="K14" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L14" s="6">
+        <f t="shared" si="13"/>
+        <v>24</v>
+      </c>
+      <c r="M14" s="7" t="str">
+        <f t="shared" ref="M14:Q14" si="15">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N14" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O14" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P14" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q14" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="4">
@@ -719,6 +1223,34 @@
       <c r="B15" s="5">
         <v>45919.0</v>
       </c>
+      <c r="K15" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L15" s="6">
+        <f t="shared" si="13"/>
+        <v>23</v>
+      </c>
+      <c r="M15" s="7" t="str">
+        <f t="shared" ref="M15:Q15" si="16">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N15" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O15" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P15" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q15" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="4">
@@ -727,6 +1259,34 @@
       <c r="B16" s="5">
         <v>45923.0</v>
       </c>
+      <c r="K16" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L16" s="6">
+        <f t="shared" si="13"/>
+        <v>24</v>
+      </c>
+      <c r="M16" s="7" t="str">
+        <f t="shared" ref="M16:Q16" si="17">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N16" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O16" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P16" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q16" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="4">
@@ -735,6 +1295,34 @@
       <c r="B17" s="5">
         <v>45925.0</v>
       </c>
+      <c r="K17" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L17" s="7" t="str">
+        <f t="shared" ref="L17:L58" si="19">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" ref="M17:M23" si="20">$J$1-$A17</f>
+        <v>22</v>
+      </c>
+      <c r="N17" s="7" t="str">
+        <f t="shared" ref="N17:Q17" si="18">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O17" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P17" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q17" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="4">
@@ -743,329 +1331,1588 @@
       <c r="B18" s="5">
         <v>45926.0</v>
       </c>
+      <c r="K18" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L18" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M18" s="6">
+        <f t="shared" si="20"/>
+        <v>24</v>
+      </c>
+      <c r="N18" s="7" t="str">
+        <f t="shared" ref="N18:Q18" si="21">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O18" s="7" t="str">
+        <f t="shared" si="21"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P18" s="7" t="str">
+        <f t="shared" si="21"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q18" s="7" t="str">
+        <f t="shared" si="21"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="7">
+      <c r="A19" s="6">
         <v>2.0</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>45930.0</v>
       </c>
+      <c r="K19" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L19" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M19" s="6">
+        <f t="shared" si="20"/>
+        <v>23</v>
+      </c>
+      <c r="N19" s="7" t="str">
+        <f t="shared" ref="N19:Q19" si="22">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O19" s="7" t="str">
+        <f t="shared" si="22"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P19" s="7" t="str">
+        <f t="shared" si="22"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q19" s="7" t="str">
+        <f t="shared" si="22"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="7">
+      <c r="A20" s="6">
         <v>2.0</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>45932.0</v>
       </c>
+      <c r="K20" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L20" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M20" s="6">
+        <f t="shared" si="20"/>
+        <v>23</v>
+      </c>
+      <c r="N20" s="7" t="str">
+        <f t="shared" ref="N20:Q20" si="23">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O20" s="7" t="str">
+        <f t="shared" si="23"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P20" s="7" t="str">
+        <f t="shared" si="23"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q20" s="7" t="str">
+        <f t="shared" si="23"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="7">
+      <c r="A21" s="6">
         <v>3.0</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="9">
         <v>45933.0</v>
+      </c>
+      <c r="K21" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L21" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M21" s="6">
+        <f t="shared" si="20"/>
+        <v>22</v>
+      </c>
+      <c r="N21" s="7" t="str">
+        <f t="shared" ref="N21:Q21" si="24">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O21" s="7" t="str">
+        <f t="shared" si="24"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P21" s="7" t="str">
+        <f t="shared" si="24"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q21" s="7" t="str">
+        <f t="shared" si="24"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1">
         <v>8.0</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="9">
         <v>45935.0</v>
       </c>
+      <c r="K22" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L22" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M22" s="6">
+        <f t="shared" si="20"/>
+        <v>17</v>
+      </c>
+      <c r="N22" s="7" t="str">
+        <f t="shared" ref="N22:Q22" si="25">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O22" s="7" t="str">
+        <f t="shared" si="25"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P22" s="7" t="str">
+        <f t="shared" si="25"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q22" s="7" t="str">
+        <f t="shared" si="25"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="7">
+      <c r="A23" s="6">
         <v>5.0</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="9">
         <v>45937.0</v>
       </c>
+      <c r="K23" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L23" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M23" s="6">
+        <f t="shared" si="20"/>
+        <v>20</v>
+      </c>
+      <c r="N23" s="7" t="str">
+        <f t="shared" ref="N23:Q23" si="26">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O23" s="7" t="str">
+        <f t="shared" si="26"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P23" s="7" t="str">
+        <f t="shared" si="26"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q23" s="7" t="str">
+        <f t="shared" si="26"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="7">
+      <c r="A24" s="6">
         <v>2.0</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="9">
         <v>45943.0</v>
       </c>
+      <c r="K24" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L24" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M24" s="7" t="str">
+        <f t="shared" ref="M24:M58" si="28">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N24" s="6">
+        <f t="shared" ref="N24:N34" si="29">$J$1-$A24</f>
+        <v>23</v>
+      </c>
+      <c r="O24" s="7" t="str">
+        <f t="shared" ref="O24:Q24" si="27">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P24" s="7" t="str">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q24" s="7" t="str">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="7">
+      <c r="A25" s="6">
         <v>4.0</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="9">
         <v>45944.0</v>
       </c>
-      <c r="G25" s="9"/>
+      <c r="G25" s="10"/>
+      <c r="K25" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L25" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M25" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N25" s="6">
+        <f t="shared" si="29"/>
+        <v>21</v>
+      </c>
+      <c r="O25" s="7" t="str">
+        <f t="shared" ref="O25:Q25" si="30">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P25" s="7" t="str">
+        <f t="shared" si="30"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q25" s="7" t="str">
+        <f t="shared" si="30"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="7">
+      <c r="A26" s="6">
         <v>1.0</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>45946.0</v>
       </c>
+      <c r="K26" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L26" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M26" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N26" s="6">
+        <f t="shared" si="29"/>
+        <v>24</v>
+      </c>
+      <c r="O26" s="7" t="str">
+        <f t="shared" ref="O26:Q26" si="31">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P26" s="7" t="str">
+        <f t="shared" si="31"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q26" s="7" t="str">
+        <f t="shared" si="31"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="7">
+      <c r="A27" s="6">
         <v>7.0</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>45947.0</v>
       </c>
+      <c r="K27" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L27" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M27" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N27" s="6">
+        <f t="shared" si="29"/>
+        <v>18</v>
+      </c>
+      <c r="O27" s="7" t="str">
+        <f t="shared" ref="O27:Q27" si="32">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P27" s="7" t="str">
+        <f t="shared" si="32"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q27" s="7" t="str">
+        <f t="shared" si="32"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="7">
+      <c r="A28" s="6">
         <v>6.0</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>45948.0</v>
       </c>
+      <c r="K28" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L28" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M28" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N28" s="6">
+        <f t="shared" si="29"/>
+        <v>19</v>
+      </c>
+      <c r="O28" s="7" t="str">
+        <f t="shared" ref="O28:Q28" si="33">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P28" s="7" t="str">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q28" s="7" t="str">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="7">
+      <c r="A29" s="6">
         <v>7.0</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>45951.0</v>
       </c>
+      <c r="K29" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L29" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M29" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N29" s="6">
+        <f t="shared" si="29"/>
+        <v>18</v>
+      </c>
+      <c r="O29" s="7" t="str">
+        <f t="shared" ref="O29:Q29" si="34">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P29" s="7" t="str">
+        <f t="shared" si="34"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q29" s="7" t="str">
+        <f t="shared" si="34"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="7">
+      <c r="A30" s="6">
         <v>1.0</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="9">
         <v>45953.0</v>
       </c>
+      <c r="K30" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L30" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M30" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N30" s="6">
+        <f t="shared" si="29"/>
+        <v>24</v>
+      </c>
+      <c r="O30" s="7" t="str">
+        <f t="shared" ref="O30:Q30" si="35">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P30" s="7" t="str">
+        <f t="shared" si="35"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q30" s="7" t="str">
+        <f t="shared" si="35"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="7">
+      <c r="A31" s="6">
         <v>3.0</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="9">
         <v>45954.0</v>
       </c>
+      <c r="K31" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L31" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M31" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N31" s="6">
+        <f t="shared" si="29"/>
+        <v>22</v>
+      </c>
+      <c r="O31" s="7" t="str">
+        <f t="shared" ref="O31:Q31" si="36">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P31" s="7" t="str">
+        <f t="shared" si="36"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q31" s="7" t="str">
+        <f t="shared" si="36"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="7">
+      <c r="A32" s="6">
         <v>6.0</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="9">
         <v>45956.0</v>
+      </c>
+      <c r="K32" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L32" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M32" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N32" s="6">
+        <f t="shared" si="29"/>
+        <v>19</v>
+      </c>
+      <c r="O32" s="7" t="str">
+        <f t="shared" ref="O32:Q32" si="37">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P32" s="7" t="str">
+        <f t="shared" si="37"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q32" s="7" t="str">
+        <f t="shared" si="37"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="3">
         <v>9.0</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="9">
         <v>45957.0</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="K33" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L33" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M33" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N33" s="3">
+        <f t="shared" si="29"/>
+        <v>16</v>
+      </c>
+      <c r="O33" s="7" t="str">
+        <f t="shared" ref="O33:Q33" si="38">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P33" s="7" t="str">
+        <f t="shared" si="38"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q33" s="7" t="str">
+        <f t="shared" si="38"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3">
         <v>5.0</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="9">
         <v>45958.0</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
+      </c>
+      <c r="K34" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L34" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M34" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N34" s="3">
+        <f t="shared" si="29"/>
+        <v>20</v>
+      </c>
+      <c r="O34" s="7" t="str">
+        <f t="shared" ref="O34:Q34" si="39">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P34" s="7" t="str">
+        <f t="shared" si="39"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q34" s="7" t="str">
+        <f t="shared" si="39"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3">
         <v>7.0</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="9">
         <v>45960.0</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
+      </c>
+      <c r="K35" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L35" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M35" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N35" s="7" t="str">
+        <f t="shared" ref="N35:N58" si="41">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O35" s="3">
+        <f t="shared" ref="O35:O43" si="42">$J$1-$A35</f>
+        <v>18</v>
+      </c>
+      <c r="P35" s="7" t="str">
+        <f t="shared" ref="P35:Q35" si="40">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q35" s="7" t="str">
+        <f t="shared" si="40"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3">
         <v>6.0</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="9">
         <v>45961.0</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="K36" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L36" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M36" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N36" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O36" s="3">
+        <f t="shared" si="42"/>
+        <v>19</v>
+      </c>
+      <c r="P36" s="7" t="str">
+        <f t="shared" ref="P36:Q36" si="43">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q36" s="7" t="str">
+        <f t="shared" si="43"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="3">
         <v>1.0</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>45962.0</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="K37" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L37" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M37" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N37" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O37" s="3">
+        <f t="shared" si="42"/>
+        <v>24</v>
+      </c>
+      <c r="P37" s="7" t="str">
+        <f t="shared" ref="P37:Q37" si="44">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q37" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="3">
         <v>1.0</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>45963.0</v>
+      </c>
+      <c r="K38" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L38" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M38" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N38" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O38" s="3">
+        <f t="shared" si="42"/>
+        <v>24</v>
+      </c>
+      <c r="P38" s="7" t="str">
+        <f t="shared" ref="P38:Q38" si="45">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q38" s="7" t="str">
+        <f t="shared" si="45"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3">
         <v>1.0</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="9">
         <v>45964.0</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K39" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L39" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M39" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N39" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O39" s="3">
+        <f t="shared" si="42"/>
+        <v>24</v>
+      </c>
+      <c r="P39" s="7" t="str">
+        <f t="shared" ref="P39:Q39" si="46">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q39" s="7" t="str">
+        <f t="shared" si="46"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3">
         <v>12.0</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="9">
         <v>45965.0</v>
+      </c>
+      <c r="D40" s="11">
+        <v>45895.0</v>
+      </c>
+      <c r="E40" s="11">
+        <f>TODAY()</f>
+        <v>45982</v>
+      </c>
+      <c r="K40" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L40" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M40" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N40" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O40" s="3">
+        <f t="shared" si="42"/>
+        <v>13</v>
+      </c>
+      <c r="P40" s="7" t="str">
+        <f t="shared" ref="P40:Q40" si="47">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q40" s="7" t="str">
+        <f t="shared" si="47"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3">
         <v>1.0</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="9">
         <v>45966.0</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E41" s="13">
+        <f>E40-D40+1</f>
+        <v>88</v>
+      </c>
+      <c r="K41" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L41" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M41" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N41" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O41" s="3">
+        <f t="shared" si="42"/>
+        <v>24</v>
+      </c>
+      <c r="P41" s="7" t="str">
+        <f t="shared" ref="P41:Q41" si="48">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q41" s="7" t="str">
+        <f t="shared" si="48"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="3">
         <v>7.0</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="9">
         <v>45967.0</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" s="13">
+        <f>COUNTA(A3:A57)</f>
+        <v>55</v>
+      </c>
+      <c r="K42" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L42" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M42" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N42" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O42" s="3">
+        <f t="shared" si="42"/>
+        <v>18</v>
+      </c>
+      <c r="P42" s="7" t="str">
+        <f t="shared" ref="P42:Q42" si="49">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q42" s="7" t="str">
+        <f t="shared" si="49"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="3">
         <v>5.0</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>45968.0</v>
+      </c>
+      <c r="D43" s="12" t="str">
+        <f>"Promedio en días totales: (" &amp; C4 &amp; "/" &amp; E41 &amp; ")"</f>
+        <v>Promedio en días totales: (307/88)</v>
+      </c>
+      <c r="E43" s="14">
+        <f>C4/E41</f>
+        <v>3.488636364</v>
+      </c>
+      <c r="K43" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L43" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M43" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N43" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O43" s="3">
+        <f t="shared" si="42"/>
+        <v>20</v>
+      </c>
+      <c r="P43" s="7" t="str">
+        <f t="shared" ref="P43:Q43" si="50">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q43" s="7" t="str">
+        <f t="shared" si="50"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3">
         <v>14.0</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="9">
         <v>45969.0</v>
+      </c>
+      <c r="D44" s="12" t="str">
+        <f>"Promedio en días efectivos: (" &amp; C4 &amp; "/" &amp; E42 &amp; ")"</f>
+        <v>Promedio en días efectivos: (307/55)</v>
+      </c>
+      <c r="E44" s="14">
+        <f>AVERAGE(A3:A57)</f>
+        <v>5.581818182</v>
+      </c>
+      <c r="K44" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L44" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M44" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N44" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O44" s="7" t="str">
+        <f t="shared" ref="O44:O58" si="51">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P44" s="3">
+        <f t="shared" ref="P44:P54" si="52">$J$1-$A44</f>
+        <v>11</v>
+      </c>
+      <c r="Q44" s="7" t="str">
+        <f t="shared" ref="Q44:Q54" si="53">$J$2</f>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="3">
         <v>7.0</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="9">
         <v>45970.0</v>
+      </c>
+      <c r="K45" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L45" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M45" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N45" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O45" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P45" s="3">
+        <f t="shared" si="52"/>
+        <v>18</v>
+      </c>
+      <c r="Q45" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="3">
         <v>13.0</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="9">
         <v>45971.0</v>
+      </c>
+      <c r="K46" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L46" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M46" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N46" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O46" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P46" s="3">
+        <f t="shared" si="52"/>
+        <v>12</v>
+      </c>
+      <c r="Q46" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="3">
         <v>21.0</v>
       </c>
-      <c r="B47" s="8">
+      <c r="B47" s="9">
         <v>45972.0</v>
+      </c>
+      <c r="K47" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L47" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M47" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N47" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O47" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P47" s="3">
+        <f t="shared" si="52"/>
+        <v>4</v>
+      </c>
+      <c r="Q47" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="3">
         <v>18.0</v>
       </c>
-      <c r="B48" s="8">
+      <c r="B48" s="9">
         <v>45973.0</v>
+      </c>
+      <c r="K48" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L48" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M48" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N48" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O48" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P48" s="3">
+        <f t="shared" si="52"/>
+        <v>7</v>
+      </c>
+      <c r="Q48" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="3">
         <v>7.0</v>
       </c>
-      <c r="B49" s="8">
+      <c r="B49" s="9">
         <v>45974.0</v>
+      </c>
+      <c r="K49" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L49" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M49" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N49" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O49" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P49" s="3">
+        <f t="shared" si="52"/>
+        <v>18</v>
+      </c>
+      <c r="Q49" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="3">
         <v>10.0</v>
       </c>
-      <c r="B50" s="8">
+      <c r="B50" s="9">
         <v>45975.0</v>
+      </c>
+      <c r="K50" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L50" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M50" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N50" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O50" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P50" s="3">
+        <f t="shared" si="52"/>
+        <v>15</v>
+      </c>
+      <c r="Q50" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="3">
         <v>8.0</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="9">
         <v>45976.0</v>
+      </c>
+      <c r="K51" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L51" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M51" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N51" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O51" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P51" s="3">
+        <f t="shared" si="52"/>
+        <v>17</v>
+      </c>
+      <c r="Q51" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="3">
         <v>7.0</v>
       </c>
-      <c r="B52" s="8">
+      <c r="B52" s="9">
         <v>45977.0</v>
+      </c>
+      <c r="K52" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L52" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M52" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N52" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O52" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P52" s="3">
+        <f t="shared" si="52"/>
+        <v>18</v>
+      </c>
+      <c r="Q52" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="3">
         <v>12.0</v>
       </c>
-      <c r="B53" s="8">
+      <c r="B53" s="9">
         <v>45978.0</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G53" s="3">
+        <v>65.0</v>
+      </c>
+      <c r="H53" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I53" s="16">
+        <f t="shared" ref="I53:I54" si="54">SUM(G53,G55)</f>
+        <v>100</v>
+      </c>
+      <c r="K53" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L53" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M53" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N53" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O53" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P53" s="3">
+        <f t="shared" si="52"/>
+        <v>13</v>
+      </c>
+      <c r="Q53" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3">
         <v>19.0</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="9">
         <v>45979.0</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" s="3">
+        <v>95.0</v>
+      </c>
+      <c r="H54" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="I54" s="16">
+        <f t="shared" si="54"/>
+        <v>171</v>
+      </c>
+      <c r="K54" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L54" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M54" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N54" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O54" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P54" s="3">
+        <f t="shared" si="52"/>
+        <v>6</v>
+      </c>
+      <c r="Q54" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3">
         <v>8.0</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="9">
         <v>45980.0</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G55" s="3">
+        <v>35.0</v>
+      </c>
+      <c r="H55" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="I55" s="15">
+        <v>35.0</v>
+      </c>
+      <c r="K55" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L55" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M55" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N55" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O55" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P55" s="7" t="str">
+        <f t="shared" ref="P55:P58" si="55">$J$2</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q55" s="3">
+        <f t="shared" ref="Q55:Q58" si="56">$J$1-$A55</f>
+        <v>17</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="3">
-        <v>11.0</v>
-      </c>
-      <c r="B56" s="8">
+        <v>13.0</v>
+      </c>
+      <c r="B56" s="9">
         <v>45981.0</v>
       </c>
-    </row>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
+      <c r="F56" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G56" s="3">
+        <v>76.0</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I56" s="13">
+        <f>SUM(G53:G57)</f>
+        <v>306</v>
+      </c>
+      <c r="K56" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L56" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M56" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N56" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O56" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P56" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q56" s="3">
+        <f t="shared" si="56"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="B57" s="9">
+        <v>45982.0</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G57" s="3">
+        <v>35.0</v>
+      </c>
+      <c r="K57" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L57" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M57" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N57" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O57" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P57" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q57" s="3">
+        <f t="shared" si="56"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="B58" s="9">
+        <v>45983.0</v>
+      </c>
+      <c r="K58" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L58" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M58" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N58" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O58" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P58" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q58" s="3">
+        <f t="shared" si="56"/>
+        <v>25</v>
+      </c>
+    </row>
     <row r="59" ht="15.75" customHeight="1"/>
     <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: actualización manuales 25-11
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="8u7A57w9g7ecO9LEvqLgIlNAKBelJsfuCUsa3Iepi5g="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="drksOt/BnM/aYUZAFyqzUs7tqeHC26RRcNZ4fBkK2W8="/>
     </ext>
   </extLst>
 </workbook>
@@ -825,7 +825,7 @@
       </c>
       <c r="C4" s="8">
         <f>SUM(A3:A80)</f>
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="K4" s="6">
         <f t="shared" si="2"/>
@@ -1116,7 +1116,7 @@
         <v>45911.0</v>
       </c>
       <c r="K12" s="7" t="str">
-        <f t="shared" ref="K12:K58" si="12">$J$2</f>
+        <f t="shared" ref="K12:K59" si="12">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="L12" s="6">
@@ -1300,7 +1300,7 @@
         <v>#N/A</v>
       </c>
       <c r="L17" s="7" t="str">
-        <f t="shared" ref="L17:L58" si="19">$J$2</f>
+        <f t="shared" ref="L17:L59" si="19">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="M17" s="6">
@@ -1556,7 +1556,7 @@
         <v>#N/A</v>
       </c>
       <c r="M24" s="7" t="str">
-        <f t="shared" ref="M24:M58" si="28">$J$2</f>
+        <f t="shared" ref="M24:M59" si="28">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="N24" s="6">
@@ -1966,7 +1966,7 @@
         <v>#N/A</v>
       </c>
       <c r="N35" s="7" t="str">
-        <f t="shared" ref="N35:N58" si="41">$J$2</f>
+        <f t="shared" ref="N35:N59" si="41">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="O35" s="3">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="E40" s="11">
         <f>TODAY()</f>
-        <v>45982</v>
+        <v>45986</v>
       </c>
       <c r="K40" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="E41" s="13">
         <f>E40-D40+1</f>
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="K41" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2276,11 +2276,11 @@
       </c>
       <c r="D43" s="12" t="str">
         <f>"Promedio en días totales: (" &amp; C4 &amp; "/" &amp; E41 &amp; ")"</f>
-        <v>Promedio en días totales: (307/88)</v>
+        <v>Promedio en días totales: (317/92)</v>
       </c>
       <c r="E43" s="14">
         <f>C4/E41</f>
-        <v>3.488636364</v>
+        <v>3.445652174</v>
       </c>
       <c r="K43" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="D44" s="12" t="str">
         <f>"Promedio en días efectivos: (" &amp; C4 &amp; "/" &amp; E42 &amp; ")"</f>
-        <v>Promedio en días efectivos: (307/55)</v>
+        <v>Promedio en días efectivos: (317/55)</v>
       </c>
       <c r="E44" s="14">
         <f>AVERAGE(A3:A57)</f>
@@ -2343,7 +2343,7 @@
         <v>#N/A</v>
       </c>
       <c r="O44" s="7" t="str">
-        <f t="shared" ref="O44:O58" si="51">$J$2</f>
+        <f t="shared" ref="O44:O59" si="51">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="P44" s="3">
@@ -2654,14 +2654,14 @@
         <v>23</v>
       </c>
       <c r="G53" s="3">
-        <v>65.0</v>
+        <v>66.0</v>
       </c>
       <c r="H53" s="15" t="s">
         <v>24</v>
       </c>
       <c r="I53" s="16">
         <f t="shared" ref="I53:I54" si="54">SUM(G53,G55)</f>
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K53" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2703,14 +2703,14 @@
         <v>25</v>
       </c>
       <c r="G54" s="3">
-        <v>95.0</v>
+        <v>102.0</v>
       </c>
       <c r="H54" s="15" t="s">
         <v>26</v>
       </c>
       <c r="I54" s="16">
         <f t="shared" si="54"/>
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="K54" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2758,7 +2758,7 @@
         <v>28</v>
       </c>
       <c r="I55" s="15">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
       <c r="K55" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2781,11 +2781,11 @@
         <v>#N/A</v>
       </c>
       <c r="P55" s="7" t="str">
-        <f t="shared" ref="P55:P58" si="55">$J$2</f>
+        <f t="shared" ref="P55:P59" si="55">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="Q55" s="3">
-        <f t="shared" ref="Q55:Q58" si="56">$J$1-$A55</f>
+        <f t="shared" ref="Q55:Q60" si="56">$J$1-$A55</f>
         <v>17</v>
       </c>
     </row>
@@ -2800,14 +2800,14 @@
         <v>29</v>
       </c>
       <c r="G56" s="3">
-        <v>76.0</v>
+        <v>78.0</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>30</v>
       </c>
       <c r="I56" s="13">
         <f>SUM(G53:G57)</f>
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="K56" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2849,7 +2849,7 @@
         <v>31</v>
       </c>
       <c r="G57" s="3">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
       <c r="K57" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2881,6 +2881,9 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="3">
+        <v>3.0</v>
+      </c>
       <c r="B58" s="9">
         <v>45983.0</v>
       </c>
@@ -2910,11 +2913,51 @@
       </c>
       <c r="Q58" s="3">
         <f t="shared" si="56"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B59" s="9">
+        <v>45986.0</v>
+      </c>
+      <c r="K59" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L59" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M59" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N59" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O59" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P59" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q59" s="3">
+        <f t="shared" si="56"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="Q60" s="3">
+        <f t="shared" si="56"/>
         <v>25</v>
       </c>
     </row>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
     <row r="63" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
actualización doc modelo de datos y avance memoria del proyecto
</commit_message>
<xml_diff>
--- a/Commmits.xlsx
+++ b/Commmits.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="drksOt/BnM/aYUZAFyqzUs7tqeHC26RRcNZ4fBkK2W8="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="dZWPvyYNZx5BJN7g+GV1A/BYpY+eTm9Ilwo7NnZhZPE="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>A</t>
   </si>
@@ -66,7 +66,13 @@
     <t>cantidad de carpetas</t>
   </si>
   <si>
+    <t>Carpetas:</t>
+  </si>
+  <si>
     <t>git rev-list --all | while read commit; do git ls-tree -r --name-only $commit; done | sed 's/[^/]*$//' | sort -u | wc -l</t>
+  </si>
+  <si>
+    <t>Archivos:</t>
   </si>
   <si>
     <t>cantidad de archivos</t>
@@ -118,10 +124,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd&quot;-&quot;mm&quot;-&quot;yy"/>
-    <numFmt numFmtId="165" formatCode="d/M/yyyy"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="166" formatCode="d/M/yyyy"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -160,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -188,14 +195,17 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="166" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="167" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -384,6 +394,13 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF">
+        <a:alpha val="0"/>
+      </a:srgbClr>
+    </a:solidFill>
+  </c:spPr>
 </c:chartSpace>
 </file>
 
@@ -825,7 +842,7 @@
       </c>
       <c r="C4" s="8">
         <f>SUM(A3:A80)</f>
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="K4" s="6">
         <f t="shared" si="2"/>
@@ -1116,7 +1133,7 @@
         <v>45911.0</v>
       </c>
       <c r="K12" s="7" t="str">
-        <f t="shared" ref="K12:K59" si="12">$J$2</f>
+        <f t="shared" ref="K12:K61" si="12">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="L12" s="6">
@@ -1300,7 +1317,7 @@
         <v>#N/A</v>
       </c>
       <c r="L17" s="7" t="str">
-        <f t="shared" ref="L17:L59" si="19">$J$2</f>
+        <f t="shared" ref="L17:L61" si="19">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="M17" s="6">
@@ -1556,7 +1573,7 @@
         <v>#N/A</v>
       </c>
       <c r="M24" s="7" t="str">
-        <f t="shared" ref="M24:M59" si="28">$J$2</f>
+        <f t="shared" ref="M24:M61" si="28">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="N24" s="6">
@@ -1875,6 +1892,12 @@
       <c r="F33" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="G33" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I33" s="11">
+        <v>45988.0</v>
+      </c>
       <c r="K33" s="7" t="str">
         <f t="shared" si="12"/>
         <v>#N/A</v>
@@ -1914,6 +1937,12 @@
       <c r="F34" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="G34" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H34" s="3">
+        <v>2367.0</v>
+      </c>
       <c r="K34" s="7" t="str">
         <f t="shared" si="12"/>
         <v>#N/A</v>
@@ -1951,7 +1980,13 @@
         <v>45960.0</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="3">
+        <v>25623.0</v>
       </c>
       <c r="K35" s="7" t="str">
         <f t="shared" si="12"/>
@@ -1966,7 +2001,7 @@
         <v>#N/A</v>
       </c>
       <c r="N35" s="7" t="str">
-        <f t="shared" ref="N35:N59" si="41">$J$2</f>
+        <f t="shared" ref="N35:N61" si="41">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="O35" s="3">
@@ -1990,7 +2025,7 @@
         <v>45961.0</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K36" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2029,7 +2064,7 @@
         <v>45962.0</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K37" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2104,10 +2139,10 @@
         <v>45964.0</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K39" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2145,12 +2180,12 @@
       <c r="B40" s="9">
         <v>45965.0</v>
       </c>
-      <c r="D40" s="11">
+      <c r="D40" s="12">
         <v>45895.0</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="12">
         <f>TODAY()</f>
-        <v>45986</v>
+        <v>45989</v>
       </c>
       <c r="K40" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2188,12 +2223,12 @@
       <c r="B41" s="9">
         <v>45966.0</v>
       </c>
-      <c r="D41" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E41" s="13">
+      <c r="D41" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" s="14">
         <f>E40-D40+1</f>
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K41" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2231,12 +2266,12 @@
       <c r="B42" s="9">
         <v>45967.0</v>
       </c>
-      <c r="D42" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E42" s="13">
-        <f>COUNTA(A3:A57)</f>
-        <v>55</v>
+      <c r="D42" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E42" s="14">
+        <f>COUNTA(A3:A61)</f>
+        <v>59</v>
       </c>
       <c r="K42" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2274,13 +2309,13 @@
       <c r="B43" s="9">
         <v>45968.0</v>
       </c>
-      <c r="D43" s="12" t="str">
+      <c r="D43" s="13" t="str">
         <f>"Promedio en días totales: (" &amp; C4 &amp; "/" &amp; E41 &amp; ")"</f>
-        <v>Promedio en días totales: (317/92)</v>
-      </c>
-      <c r="E43" s="14">
+        <v>Promedio en días totales: (327/95)</v>
+      </c>
+      <c r="E43" s="15">
         <f>C4/E41</f>
-        <v>3.445652174</v>
+        <v>3.442105263</v>
       </c>
       <c r="K43" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2318,11 +2353,11 @@
       <c r="B44" s="9">
         <v>45969.0</v>
       </c>
-      <c r="D44" s="12" t="str">
+      <c r="D44" s="13" t="str">
         <f>"Promedio en días efectivos: (" &amp; C4 &amp; "/" &amp; E42 &amp; ")"</f>
-        <v>Promedio en días efectivos: (317/55)</v>
-      </c>
-      <c r="E44" s="14">
+        <v>Promedio en días efectivos: (327/59)</v>
+      </c>
+      <c r="E44" s="15">
         <f>AVERAGE(A3:A57)</f>
         <v>5.581818182</v>
       </c>
@@ -2343,7 +2378,7 @@
         <v>#N/A</v>
       </c>
       <c r="O44" s="7" t="str">
-        <f t="shared" ref="O44:O59" si="51">$J$2</f>
+        <f t="shared" ref="O44:O61" si="51">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="P44" s="3">
@@ -2651,17 +2686,17 @@
         <v>45978.0</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G53" s="3">
-        <v>66.0</v>
-      </c>
-      <c r="H53" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="I53" s="16">
+        <v>67.0</v>
+      </c>
+      <c r="H53" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="I53" s="17">
         <f t="shared" ref="I53:I54" si="54">SUM(G53,G55)</f>
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K53" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2700,17 +2735,17 @@
         <v>45979.0</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G54" s="3">
-        <v>102.0</v>
-      </c>
-      <c r="H54" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="I54" s="16">
+        <v>106.0</v>
+      </c>
+      <c r="H54" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I54" s="17">
         <f t="shared" si="54"/>
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="K54" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2749,16 +2784,17 @@
         <v>45980.0</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G55" s="3">
         <v>35.0</v>
       </c>
-      <c r="H55" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="I55" s="15">
-        <v>36.0</v>
+      <c r="H55" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I55" s="16">
+        <f>G57</f>
+        <v>40</v>
       </c>
       <c r="K55" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2781,11 +2817,11 @@
         <v>#N/A</v>
       </c>
       <c r="P55" s="7" t="str">
-        <f t="shared" ref="P55:P59" si="55">$J$2</f>
+        <f t="shared" ref="P55:P61" si="55">$J$2</f>
         <v>#N/A</v>
       </c>
       <c r="Q55" s="3">
-        <f t="shared" ref="Q55:Q60" si="56">$J$1-$A55</f>
+        <f t="shared" ref="Q55:Q61" si="56">$J$1-$A55</f>
         <v>17</v>
       </c>
     </row>
@@ -2797,17 +2833,17 @@
         <v>45981.0</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G56" s="3">
-        <v>78.0</v>
+        <v>79.0</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I56" s="13">
+        <v>32</v>
+      </c>
+      <c r="I56" s="14">
         <f>SUM(G53:G57)</f>
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="K56" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2846,10 +2882,10 @@
         <v>45982.0</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G57" s="3">
-        <v>36.0</v>
+        <v>40.0</v>
       </c>
       <c r="K57" s="7" t="str">
         <f t="shared" si="12"/>
@@ -2918,7 +2954,7 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="3">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="B59" s="9">
         <v>45986.0</v>
@@ -2949,16 +2985,81 @@
       </c>
       <c r="Q59" s="3">
         <f t="shared" si="56"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B60" s="9">
+        <v>45988.0</v>
+      </c>
+      <c r="K60" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L60" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M60" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N60" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O60" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P60" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
       <c r="Q60" s="3">
         <f t="shared" si="56"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="61" ht="15.75" customHeight="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B61" s="9">
+        <v>45989.0</v>
+      </c>
+      <c r="K61" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L61" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M61" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N61" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O61" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P61" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>#N/A</v>
+      </c>
+      <c r="Q61" s="3">
+        <f t="shared" si="56"/>
+        <v>18</v>
+      </c>
+    </row>
     <row r="62" ht="15.75" customHeight="1"/>
     <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1"/>

</xml_diff>